<commit_message>
test: local run as the submitted evidence, with the console screenshot section 11 names
Port 3000 was freed (the other project's kind cluster was stopped with the student's approval), so the
submitted reports are now a local run against localhost:3000 rather than CI artefacts: 29/30/30 and the
regression suite 216/0, identical to the runner. Seven runs across two operating systems now agree.

--reporter-htmlextra-logs puts the pre-request script's console.log into the report, so section 11's
'console screenshot from your pre-request script' is satisfied by an artefact of the run itself:
console-x-student-id.png shows CONSOLE LOGS printing
[HW06] X-Student-Id =23127178|POST/api/login|2026-08-22T15:17:35.271Z.
The flag is now the default in both the local runner and the workflow, so the evidence regenerates with
every run instead of depending on a one-off capture.
</commit_message>
<xml_diff>
--- a/excel/23127178_HW06_TestCases.xlsx
+++ b/excel/23127178_HW06_TestCases.xlsx
@@ -9432,7 +9432,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-22T15:00:11.332Z</t>
+          <t>2026-08-22T15:17:35.263Z</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -9462,7 +9462,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>1.1s</t>
+          <t>0.8s</t>
         </is>
       </c>
     </row>
@@ -9474,7 +9474,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-22T15:00:13.645Z</t>
+          <t>2026-08-22T15:17:37.764Z</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -9504,7 +9504,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>1.0s</t>
+          <t>0.9s</t>
         </is>
       </c>
     </row>
@@ -9516,7 +9516,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-22T15:00:16.102Z</t>
+          <t>2026-08-22T15:17:41.396Z</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>1.1s</t>
+          <t>0.8s</t>
         </is>
       </c>
     </row>
@@ -9580,7 +9580,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>**3.2s**</t>
+          <t>**2.5s**</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: record the student's own verification run as the submitted evidence
The submitted reports are now the run the student executed themselves (23/08 00:09): 29/30/30 across the
three collections plus 216/0 on the regression suite, identical to every earlier run. That is a better
provenance than a run produced during the authoring session.

Human review is filled in only for what was actually verified, with the scope written down: three of the
nineteen bugs reproduced by hand (BUG-08, BUG-13, BUG-14 - the Critical ones), the full suite re-run, and
the Postman GUI console capture. Six interactions still say 'not yet checked by the student' because they
depend on reading the three audit.md files, and marking those would be exactly the manufactured evidence
section 11 penalises.
</commit_message>
<xml_diff>
--- a/excel/23127178_HW06_TestCases.xlsx
+++ b/excel/23127178_HW06_TestCases.xlsx
@@ -9432,7 +9432,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>2026-08-22T15:17:35.263Z</t>
+          <t>2026-08-22T17:09:50.309Z</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -9462,7 +9462,7 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>0.8s</t>
+          <t>0.9s</t>
         </is>
       </c>
     </row>
@@ -9474,7 +9474,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>2026-08-22T15:17:37.764Z</t>
+          <t>2026-08-22T17:09:52.873Z</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -9504,7 +9504,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>0.9s</t>
+          <t>0.8s</t>
         </is>
       </c>
     </row>
@@ -9516,7 +9516,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-08-22T15:17:41.396Z</t>
+          <t>2026-08-22T17:09:55.804Z</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -9546,7 +9546,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>0.8s</t>
+          <t>1.0s</t>
         </is>
       </c>
     </row>
@@ -9580,7 +9580,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>**2.5s**</t>
+          <t>**2.6s**</t>
         </is>
       </c>
     </row>

</xml_diff>